<commit_message>
made a few adjustment
</commit_message>
<xml_diff>
--- a/PaymentTerms.xlsx
+++ b/PaymentTerms.xlsx
@@ -24,12 +24,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="162">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Due Date</t>
   </si>
   <si>
     <t xml:space="preserve">Net 30</t>
@@ -809,7 +812,9 @@
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4"/>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
@@ -836,12 +841,14 @@
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
@@ -868,12 +875,14 @@
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="4"/>
+      <c r="C3" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
@@ -900,12 +909,14 @@
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="C4" s="4"/>
+      <c r="C4" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
@@ -932,12 +943,14 @@
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="C5" s="4"/>
+      <c r="C5" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
@@ -964,12 +977,14 @@
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="C6" s="4"/>
+      <c r="C6" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
@@ -996,12 +1011,14 @@
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="C7" s="4"/>
+      <c r="C7" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
@@ -7772,7 +7789,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>1</v>
@@ -7803,10 +7820,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>1</v>
@@ -7837,10 +7854,10 @@
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>2</v>
@@ -14750,10 +14767,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>0</v>
@@ -14786,13 +14803,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>1</v>
@@ -14822,13 +14839,13 @@
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>2</v>
@@ -14858,13 +14875,13 @@
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>3</v>
@@ -14894,13 +14911,13 @@
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>4</v>
@@ -14930,13 +14947,13 @@
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>5</v>
@@ -14966,13 +14983,13 @@
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>6</v>
@@ -15002,13 +15019,13 @@
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>7</v>
@@ -15038,13 +15055,13 @@
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>8</v>
@@ -15074,13 +15091,13 @@
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>9</v>
@@ -15110,13 +15127,13 @@
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>10</v>
@@ -15146,13 +15163,13 @@
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>11</v>
@@ -15182,13 +15199,13 @@
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>12</v>
@@ -15218,13 +15235,13 @@
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>13</v>
@@ -15254,13 +15271,13 @@
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>14</v>
@@ -15290,13 +15307,13 @@
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>15</v>
@@ -15326,13 +15343,13 @@
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>16</v>
@@ -15362,13 +15379,13 @@
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D18" s="3" t="n">
         <v>17</v>
@@ -15398,13 +15415,13 @@
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D19" s="3" t="n">
         <v>18</v>
@@ -15434,13 +15451,13 @@
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D20" s="3" t="n">
         <v>19</v>
@@ -15470,13 +15487,13 @@
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D21" s="3" t="n">
         <v>20</v>
@@ -15506,13 +15523,13 @@
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D22" s="3" t="n">
         <v>21</v>
@@ -15542,13 +15559,13 @@
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D23" s="3" t="n">
         <v>22</v>
@@ -15578,13 +15595,13 @@
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D24" s="3" t="n">
         <v>23</v>
@@ -15614,13 +15631,13 @@
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D25" s="3" t="n">
         <v>24</v>
@@ -15650,13 +15667,13 @@
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D26" s="3" t="n">
         <v>25</v>
@@ -15686,13 +15703,13 @@
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D27" s="3" t="n">
         <v>26</v>
@@ -15722,13 +15739,13 @@
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D28" s="3" t="n">
         <v>27</v>
@@ -15758,13 +15775,13 @@
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D29" s="3" t="n">
         <v>28</v>
@@ -15794,13 +15811,13 @@
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D30" s="3" t="n">
         <v>29</v>
@@ -15830,13 +15847,13 @@
     </row>
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D31" s="3" t="n">
         <v>30</v>
@@ -15866,13 +15883,13 @@
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D32" s="3" t="n">
         <v>31</v>
@@ -15902,13 +15919,13 @@
     </row>
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D33" s="3" t="n">
         <v>32</v>
@@ -15938,13 +15955,13 @@
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D34" s="3" t="n">
         <v>33</v>
@@ -15974,13 +15991,13 @@
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D35" s="3" t="n">
         <v>34</v>
@@ -16010,13 +16027,13 @@
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D36" s="3" t="n">
         <v>35</v>
@@ -16046,13 +16063,13 @@
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D37" s="3" t="n">
         <v>36</v>
@@ -16082,13 +16099,13 @@
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D38" s="3" t="n">
         <v>37</v>
@@ -16118,13 +16135,13 @@
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D39" s="3" t="n">
         <v>38</v>
@@ -16154,13 +16171,13 @@
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D40" s="3" t="n">
         <v>39</v>
@@ -16190,13 +16207,13 @@
     </row>
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D41" s="3" t="n">
         <v>40</v>
@@ -16226,13 +16243,13 @@
     </row>
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D42" s="3" t="n">
         <v>41</v>
@@ -16262,13 +16279,13 @@
     </row>
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D43" s="3" t="n">
         <v>42</v>
@@ -16298,13 +16315,13 @@
     </row>
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D44" s="3" t="n">
         <v>43</v>
@@ -16334,13 +16351,13 @@
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D45" s="3" t="n">
         <v>44</v>
@@ -16370,13 +16387,13 @@
     </row>
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D46" s="3" t="n">
         <v>45</v>
@@ -16406,13 +16423,13 @@
     </row>
     <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D47" s="3" t="n">
         <v>46</v>
@@ -16442,13 +16459,13 @@
     </row>
     <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D48" s="3" t="n">
         <v>47</v>
@@ -16478,13 +16495,13 @@
     </row>
     <row r="49" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D49" s="3" t="n">
         <v>48</v>
@@ -16514,13 +16531,13 @@
     </row>
     <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D50" s="3" t="n">
         <v>49</v>
@@ -16550,13 +16567,13 @@
     </row>
     <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D51" s="3" t="n">
         <v>50</v>
@@ -16586,13 +16603,13 @@
     </row>
     <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D52" s="3" t="n">
         <v>51</v>
@@ -16622,13 +16639,13 @@
     </row>
     <row r="53" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D53" s="3" t="n">
         <v>52</v>
@@ -16658,13 +16675,13 @@
     </row>
     <row r="54" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D54" s="3" t="n">
         <v>53</v>
@@ -16694,13 +16711,13 @@
     </row>
     <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D55" s="3" t="n">
         <v>54</v>
@@ -16730,13 +16747,13 @@
     </row>
     <row r="56" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D56" s="3" t="n">
         <v>55</v>
@@ -16766,13 +16783,13 @@
     </row>
     <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D57" s="3" t="n">
         <v>56</v>
@@ -16802,13 +16819,13 @@
     </row>
     <row r="58" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D58" s="3" t="n">
         <v>57</v>
@@ -16838,13 +16855,13 @@
     </row>
     <row r="59" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D59" s="3" t="n">
         <v>58</v>
@@ -16874,13 +16891,13 @@
     </row>
     <row r="60" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D60" s="3" t="n">
         <v>59</v>
@@ -16910,13 +16927,13 @@
     </row>
     <row r="61" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D61" s="3" t="n">
         <v>60</v>
@@ -16946,13 +16963,13 @@
     </row>
     <row r="62" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D62" s="3" t="n">
         <v>61</v>
@@ -16982,13 +16999,13 @@
     </row>
     <row r="63" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D63" s="3" t="n">
         <v>62</v>
@@ -17018,13 +17035,13 @@
     </row>
     <row r="64" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D64" s="3" t="n">
         <v>63</v>
@@ -17054,13 +17071,13 @@
     </row>
     <row r="65" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D65" s="3" t="n">
         <v>64</v>
@@ -23457,7 +23474,7 @@
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B2" s="3" t="n">
         <v>1</v>
@@ -23465,7 +23482,7 @@
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>2</v>
@@ -23473,7 +23490,7 @@
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>3</v>
@@ -23481,7 +23498,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>4</v>
@@ -25160,62 +25177,62 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B2" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>